<commit_message>
fix(pfos): teklif gorsellerini Stok no sutunu hizasina al
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
+++ b/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
@@ -221,9 +221,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -735,18 +733,18 @@
       </c>
     </row>
     <row r="7" ht="120" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>28</v>
-      </c>
+      <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="11" t="s">
+      <c r="D7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>29</v>
       </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
       <c r="I7" s="11"/>
       <c r="J7" s="11"/>
       <c r="K7" s="11"/>
@@ -1027,8 +1025,8 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="H7:M7"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="E7:M7"/>
     <mergeCell ref="A22:M22"/>
     <mergeCell ref="A23:M23"/>
     <mergeCell ref="A24:M24"/>

</xml_diff>

<commit_message>
ui(pfos): proforma tablo duzeni — EK kaldir, marka/olcu saga, tanim genis
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
+++ b/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
   <si>
     <t>PROFORMA FATURA</t>
   </si>
@@ -43,34 +43,31 @@
     <t>Poz</t>
   </si>
   <si>
-    <t>EK</t>
-  </si>
-  <si>
     <t>Stok no</t>
   </si>
   <si>
     <t>Tanımı</t>
   </si>
   <si>
+    <t>Elk. kW</t>
+  </si>
+  <si>
+    <t>Gaz kW</t>
+  </si>
+  <si>
+    <t>Adet</t>
+  </si>
+  <si>
+    <t>Satış</t>
+  </si>
+  <si>
+    <t>Toplam</t>
+  </si>
+  <si>
     <t>Marka</t>
   </si>
   <si>
     <t>Ölçü</t>
-  </si>
-  <si>
-    <t>Elk. kW</t>
-  </si>
-  <si>
-    <t>Gaz kW</t>
-  </si>
-  <si>
-    <t>Adet</t>
-  </si>
-  <si>
-    <t>Satış</t>
-  </si>
-  <si>
-    <t>Toplam</t>
   </si>
   <si>
     <t>Döviz</t>
@@ -206,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -219,8 +216,14 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -574,21 +577,19 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="4" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="9" width="8" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="6" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -633,7 +634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
@@ -670,13 +671,10 @@
       <c r="L4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="M4" s="5" t="s">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>21</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -689,274 +687,256 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>23</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>3</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="F6" s="9">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7">
+        <v>1</v>
+      </c>
+      <c r="H6" s="10">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="10">
+        <f>G6*H6</f>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="8">
-        <v>3.5</v>
-      </c>
-      <c r="I6" s="8">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7">
-        <v>1</v>
-      </c>
-      <c r="K6" s="9">
-        <v>1000</v>
-      </c>
-      <c r="L6" s="9">
-        <f>J6*K6</f>
-      </c>
-      <c r="M6" s="7" t="s">
+    </row>
+    <row r="7" ht="120" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="13" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" ht="120" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="15" t="s">
-        <v>31</v>
-      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="14"/>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="13" t="s">
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="18"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="K14" s="12"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="12"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="12"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
-      <c r="M20" s="12"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -969,11 +949,10 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -986,11 +965,10 @@
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1003,11 +981,10 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1020,17 +997,16 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="E7:M7"/>
-    <mergeCell ref="A22:M22"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="A24:M24"/>
-    <mergeCell ref="A25:M25"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="D7:L7"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A25:L25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
fix(teklif-v14): shift description column; round totals
Ürün açıklaması satırı Excel'de bir sütun sağa kaydırıldı. Satış/Toplam ve dip genel toplamda kuruşlar kaldırılıp tam sayıya yuvarlandı.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
+++ b/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
@@ -220,7 +220,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -234,7 +234,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -732,10 +732,10 @@
       <c r="C7" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="12"/>
+      <c r="E7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
@@ -1002,7 +1002,7 @@
   <mergeCells count="7">
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="D7:L7"/>
+    <mergeCell ref="E7:L7"/>
     <mergeCell ref="A22:L22"/>
     <mergeCell ref="A23:L23"/>
     <mergeCell ref="A24:L24"/>

</xml_diff>

<commit_message>
feat(pfos): improve bain-marie/banket matching and update cafe category templates
</commit_message>
<xml_diff>
--- a/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
+++ b/E-TICARET/site/public/data/templates/equsto_teklif_v14.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t>PROFORMA FATURA</t>
   </si>
@@ -102,9 +102,6 @@
   </si>
   <si>
     <t>Gazlı cihaz toplam bağlantısı (kW)</t>
-  </si>
-  <si>
-    <t>Sütun toplamları →</t>
   </si>
   <si>
     <t>GENEL TOPLAM</t>
@@ -821,7 +818,7 @@
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
       <c r="D13" s="17" t="s">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
@@ -841,7 +838,7 @@
       <c r="F14" s="14"/>
       <c r="G14" s="14"/>
       <c r="H14" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I14" s="18"/>
       <c r="J14" s="14"/>
@@ -936,7 +933,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -952,7 +949,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -968,7 +965,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -984,7 +981,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>

</xml_diff>